<commit_message>
feat: Addto cart & checkout functionality test
</commit_message>
<xml_diff>
--- a/sauce-demo/src/test/resources/testdata/cart_items.xlsx
+++ b/sauce-demo/src/test/resources/testdata/cart_items.xlsx
@@ -20,24 +20,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t xml:space="preserve">productName</t>
-  </si>
-  <si>
-    <t xml:space="preserve">testType</t>
   </si>
   <si>
     <t xml:space="preserve">Sauce Labs Backpack </t>
   </si>
   <si>
-    <t xml:space="preserve">smoke </t>
-  </si>
-  <si>
     <t xml:space="preserve">Sauce Labs Bike Light </t>
-  </si>
-  <si>
-    <t xml:space="preserve">regression </t>
   </si>
   <si>
     <t xml:space="preserve">Sauce Labs Bolt T-Shirt </t>
@@ -152,7 +143,7 @@
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="3" style="0" width="8.45"/>
   </cols>
   <sheetData>
@@ -160,49 +151,37 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2" s="1"/>
     </row>
-    <row r="2" customFormat="false" ht="25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="B4" s="1"/>
     </row>
-    <row r="3" customFormat="false" ht="25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B5" s="1"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>5</v>
-      </c>
+      <c r="B6" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>